<commit_message>
tested with more data
</commit_message>
<xml_diff>
--- a/presentation/Παρουσίαση εργασίας 2.xlsx
+++ b/presentation/Παρουσίαση εργασίας 2.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yiann\OneDrive\Υπολογιστής\Σχολείο\ΟΠΑ\Δομές δεδομένων\Εργασία 2\presentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAD4EF2F-E940-489F-9AA7-1C83E0E62753}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D7AEDF6-A4C7-482A-8E3C-8A3C9A1C166D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Φύλλο1" sheetId="1" r:id="rId1"/>
+    <sheet name="Linear data" sheetId="1" r:id="rId1"/>
+    <sheet name="Logarithmic data" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="5">
   <si>
     <t>Number of Folders</t>
   </si>
@@ -50,7 +51,7 @@
     <t>Precentile difference</t>
   </si>
   <si>
-    <t>Difference</t>
+    <t>Difference from greedy to greedy decreasing algorithm</t>
   </si>
 </sst>
 </file>
@@ -200,7 +201,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Φύλλο1!$A$2</c:f>
+              <c:f>'Linear data'!$A$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -281,7 +282,7 @@
           </c:dLbls>
           <c:cat>
             <c:numRef>
-              <c:f>Φύλλο1!$B$1:$K$1</c:f>
+              <c:f>'Linear data'!$B$1:$K$1</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -320,7 +321,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Φύλλο1!$B$2:$K$2</c:f>
+              <c:f>'Linear data'!$B$2:$K$2</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -369,7 +370,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Φύλλο1!$A$3</c:f>
+              <c:f>'Linear data'!$A$3</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -538,7 +539,7 @@
           </c:dLbls>
           <c:cat>
             <c:numRef>
-              <c:f>Φύλλο1!$B$1:$K$1</c:f>
+              <c:f>'Linear data'!$B$1:$K$1</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -577,7 +578,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Φύλλο1!$B$3:$K$3</c:f>
+              <c:f>'Linear data'!$B$3:$K$3</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -1028,7 +1029,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>Φύλλο1!$B$1:$K$1</c:f>
+              <c:f>'Linear data'!$B$1:$K$1</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -1067,39 +1068,39 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Φύλλο1!$B$4:$K$4</c:f>
+              <c:f>'Linear data'!$B$4:$K$4</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>6.1999999999999957</c:v>
+                  <c:v>-6.1999999999999957</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>21.699999999999989</c:v>
+                  <c:v>-21.699999999999989</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>36.800000000000011</c:v>
+                  <c:v>-36.800000000000011</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>53.5</c:v>
+                  <c:v>-53.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>68.700000000000045</c:v>
+                  <c:v>-68.700000000000045</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>85.699999999999932</c:v>
+                  <c:v>-85.699999999999932</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>102</c:v>
+                  <c:v>-102</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>116.34999999999991</c:v>
+                  <c:v>-116.34999999999991</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>134.25</c:v>
+                  <c:v>-134.25</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>152.5</c:v>
+                  <c:v>-152.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1484,7 +1485,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Φύλλο1!$B$1:$K$1</c:f>
+              <c:f>'Linear data'!$B$1:$K$1</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -1523,39 +1524,39 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Φύλλο1!$B$5:$K$5</c:f>
+              <c:f>'Linear data'!$B$5:$K$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>12</c:v>
+                  <c:v>-11</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>14.000000000000002</c:v>
+                  <c:v>-12</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>14.000000000000002</c:v>
+                  <c:v>-13</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>15</c:v>
+                  <c:v>-13</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>15</c:v>
+                  <c:v>-13</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>15</c:v>
+                  <c:v>-13</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>15</c:v>
+                  <c:v>-13</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>15</c:v>
+                  <c:v>-13</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>16</c:v>
+                  <c:v>-13</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>16</c:v>
+                  <c:v>-14.000000000000002</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1564,6 +1565,1743 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-9DE0-487C-9535-C707D4CC9049}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:smooth val="0"/>
+        <c:axId val="1485362208"/>
+        <c:axId val="1485362624"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="1485362208"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Number of folders</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1485362624"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1485362624"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>% difference</a:t>
+                </a:r>
+                <a:endParaRPr lang="el-GR"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1485362208"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="el-GR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Disks</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> used by algorithm</a:t>
+            </a:r>
+            <a:endParaRPr lang="el-GR"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="7.4885529819721436E-2"/>
+          <c:y val="0.11557971014492753"/>
+          <c:w val="0.90425941282887079"/>
+          <c:h val="0.66086161676808042"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Logarithmic data'!$A$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Greedy Algorithm</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="t"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:numRef>
+              <c:f>'Logarithmic data'!$B$1:$K$1</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>300</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>500</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>700</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>900</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1100</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1300</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1500</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1700</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1900</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Logarithmic data'!$B$2:$K$2</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>58.8</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>177.7</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>293.75</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>411.2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>528.45000000000005</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>646.29999999999995</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>762.25</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>881.3</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>995.55</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1105.3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-0FF1-4E74-A1A5-9B44EC70D1EA}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Logarithmic data'!$A$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Greedy Decreasing Algorithm</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="0"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="4.4618217468100365E-4"/>
+                  <c:y val="1.4593246242070085E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000001-0FF1-4E74-A1A5-9B44EC70D1EA}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-2.3116602957219044E-2"/>
+                  <c:y val="2.4305931748627423E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000002-0FF1-4E74-A1A5-9B44EC70D1EA}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="2"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-2.2081241996521964E-2"/>
+                  <c:y val="1.7830808077589317E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000003-0FF1-4E74-A1A5-9B44EC70D1EA}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="3"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-8.7034177963922002E-3"/>
+                  <c:y val="2.1068369913108429E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000004-0FF1-4E74-A1A5-9B44EC70D1EA}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="t"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:numRef>
+              <c:f>'Logarithmic data'!$B$1:$K$1</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>300</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>500</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>700</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>900</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1100</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1300</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1500</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1700</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1900</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Logarithmic data'!$B$3:$K$3</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>52.6</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>156</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>256.95</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>357.7</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>459.75</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>560.6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>660.25</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>764.95</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>861.3</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>952.8</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000005-0FF1-4E74-A1A5-9B44EC70D1EA}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:smooth val="0"/>
+        <c:axId val="1128517408"/>
+        <c:axId val="1128517824"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="1128517408"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Number of folders</a:t>
+                </a:r>
+                <a:endParaRPr lang="el-GR"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1128517824"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1128517824"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Disks</a:t>
+                </a:r>
+                <a:endParaRPr lang="el-GR"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="5.2137643378519288E-3"/>
+              <c:y val="0.43446412083865016"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1128517408"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="el-GR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t>Absolut difference in disk usage between algorithms</a:t>
+            </a:r>
+            <a:endParaRPr lang="el-GR"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:numRef>
+              <c:f>'Logarithmic data'!$B$1:$K$1</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>300</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>500</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>700</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>900</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1100</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1300</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1500</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1700</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1900</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Logarithmic data'!$B$4:$K$4</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>-6.1999999999999957</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-21.699999999999989</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-36.800000000000011</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-53.5</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-68.700000000000045</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-85.699999999999932</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-102</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-116.34999999999991</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-134.25</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-152.5</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-5922-4D3C-906F-93F14BB2645B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="769286656"/>
+        <c:axId val="769291648"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="769286656"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Number of folders</a:t>
+                </a:r>
+                <a:endParaRPr lang="el-GR"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="769291648"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="769291648"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Difference in disks</a:t>
+                </a:r>
+                <a:endParaRPr lang="el-GR"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="769286656"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="el-GR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Precentile</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> difference in disk usage</a:t>
+            </a:r>
+            <a:endParaRPr lang="el-GR"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>'Logarithmic data'!$B$1:$K$1</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>300</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>500</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>700</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>900</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1100</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1300</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1500</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1700</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1900</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Logarithmic data'!$B$5:$K$5</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>-11</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-12</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-13</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-13</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-13</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-13</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-13</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-13</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-13</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-14.000000000000002</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-8CFD-440A-BF71-36313057CAF0}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1956,6 +3694,120 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="12">
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="12">
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors6.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
   <cs:axisTitle>
@@ -2976,6 +4828,1541 @@
 </file>
 
 <file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style6.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -3532,15 +6919,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>23813</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>16124</xdr:rowOff>
+      <xdr:rowOff>28030</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>594360</xdr:colOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>10954</xdr:colOff>
       <xdr:row>25</xdr:row>
-      <xdr:rowOff>154780</xdr:rowOff>
+      <xdr:rowOff>166686</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3588,6 +6975,125 @@
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>601489</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>593869</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Γράφημα 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3383839C-0A50-40C3-9AE1-E7B8B57A57F9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>23813</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>28030</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>10954</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>166686</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Γράφημα 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2C6D35AD-3E91-42CF-ABE8-6C06B2429B14}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>767</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>270717</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>11906</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Γράφημα 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{697A70FF-4AAE-4C3D-9B22-EAFE069AA790}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="0"/>
@@ -3870,7 +7376,7 @@
   <dimension ref="A1:K5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="54.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3984,44 +7490,44 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <f>B2-B3</f>
-        <v>6.1999999999999957</v>
+        <f>B3-B2</f>
+        <v>-6.1999999999999957</v>
       </c>
       <c r="C4">
-        <f t="shared" ref="C4:E4" si="0">C2-C3</f>
-        <v>21.699999999999989</v>
+        <f t="shared" ref="C4:K4" si="0">C3-C2</f>
+        <v>-21.699999999999989</v>
       </c>
       <c r="D4">
         <f t="shared" si="0"/>
-        <v>36.800000000000011</v>
+        <v>-36.800000000000011</v>
       </c>
       <c r="E4">
         <f t="shared" si="0"/>
-        <v>53.5</v>
+        <v>-53.5</v>
       </c>
       <c r="F4">
-        <f t="shared" ref="F4" si="1">F2-F3</f>
-        <v>68.700000000000045</v>
+        <f t="shared" si="0"/>
+        <v>-68.700000000000045</v>
       </c>
       <c r="G4">
-        <f t="shared" ref="G4" si="2">G2-G3</f>
-        <v>85.699999999999932</v>
+        <f t="shared" si="0"/>
+        <v>-85.699999999999932</v>
       </c>
       <c r="H4">
-        <f t="shared" ref="H4" si="3">H2-H3</f>
-        <v>102</v>
+        <f t="shared" si="0"/>
+        <v>-102</v>
       </c>
       <c r="I4">
-        <f t="shared" ref="I4" si="4">I2-I3</f>
-        <v>116.34999999999991</v>
+        <f t="shared" si="0"/>
+        <v>-116.34999999999991</v>
       </c>
       <c r="J4">
-        <f t="shared" ref="J4" si="5">J2-J3</f>
-        <v>134.25</v>
+        <f t="shared" si="0"/>
+        <v>-134.25</v>
       </c>
       <c r="K4">
-        <f t="shared" ref="K4" si="6">K2-K3</f>
-        <v>152.5</v>
+        <f t="shared" si="0"/>
+        <v>-152.5</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
@@ -4029,44 +7535,254 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <f>ROUND(B4/B3, 2) * 100</f>
-        <v>12</v>
+        <f>(ROUND(B4/B2, 2) * 100)</f>
+        <v>-11</v>
       </c>
       <c r="C5">
-        <f t="shared" ref="C5:E5" si="7">ROUND(C4/C3, 2) * 100</f>
-        <v>14.000000000000002</v>
+        <f t="shared" ref="C5:K5" si="1">(ROUND(C4/C2, 2) * 100)</f>
+        <v>-12</v>
       </c>
       <c r="D5">
-        <f t="shared" si="7"/>
-        <v>14.000000000000002</v>
+        <f t="shared" si="1"/>
+        <v>-13</v>
       </c>
       <c r="E5">
-        <f t="shared" si="7"/>
-        <v>15</v>
+        <f t="shared" si="1"/>
+        <v>-13</v>
       </c>
       <c r="F5">
-        <f t="shared" ref="F5" si="8">ROUND(F4/F3, 2) * 100</f>
-        <v>15</v>
+        <f t="shared" si="1"/>
+        <v>-13</v>
       </c>
       <c r="G5">
-        <f t="shared" ref="G5" si="9">ROUND(G4/G3, 2) * 100</f>
-        <v>15</v>
+        <f t="shared" si="1"/>
+        <v>-13</v>
       </c>
       <c r="H5">
-        <f t="shared" ref="H5" si="10">ROUND(H4/H3, 2) * 100</f>
-        <v>15</v>
+        <f t="shared" si="1"/>
+        <v>-13</v>
       </c>
       <c r="I5">
-        <f t="shared" ref="I5" si="11">ROUND(I4/I3, 2) * 100</f>
-        <v>15</v>
+        <f t="shared" si="1"/>
+        <v>-13</v>
       </c>
       <c r="J5">
-        <f t="shared" ref="J5" si="12">ROUND(J4/J3, 2) * 100</f>
-        <v>16</v>
+        <f t="shared" si="1"/>
+        <v>-13</v>
       </c>
       <c r="K5">
-        <f t="shared" ref="K5" si="13">ROUND(K4/K3, 2) * 100</f>
-        <v>16</v>
+        <f t="shared" si="1"/>
+        <v>-14.000000000000002</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8247851E-4746-47B1-81A1-0680B06091CD}">
+  <dimension ref="A1:K5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="54.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1">
+        <v>100</v>
+      </c>
+      <c r="C1">
+        <v>300</v>
+      </c>
+      <c r="D1">
+        <v>500</v>
+      </c>
+      <c r="E1">
+        <v>700</v>
+      </c>
+      <c r="F1">
+        <v>900</v>
+      </c>
+      <c r="G1">
+        <v>1100</v>
+      </c>
+      <c r="H1">
+        <v>1300</v>
+      </c>
+      <c r="I1">
+        <v>1500</v>
+      </c>
+      <c r="J1">
+        <v>1700</v>
+      </c>
+      <c r="K1">
+        <v>1900</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2">
+        <v>58.8</v>
+      </c>
+      <c r="C2">
+        <v>177.7</v>
+      </c>
+      <c r="D2">
+        <v>293.75</v>
+      </c>
+      <c r="E2">
+        <v>411.2</v>
+      </c>
+      <c r="F2">
+        <v>528.45000000000005</v>
+      </c>
+      <c r="G2">
+        <v>646.29999999999995</v>
+      </c>
+      <c r="H2">
+        <v>762.25</v>
+      </c>
+      <c r="I2">
+        <v>881.3</v>
+      </c>
+      <c r="J2">
+        <v>995.55</v>
+      </c>
+      <c r="K2">
+        <v>1105.3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>52.6</v>
+      </c>
+      <c r="C3">
+        <v>156</v>
+      </c>
+      <c r="D3">
+        <v>256.95</v>
+      </c>
+      <c r="E3">
+        <v>357.7</v>
+      </c>
+      <c r="F3">
+        <v>459.75</v>
+      </c>
+      <c r="G3">
+        <v>560.6</v>
+      </c>
+      <c r="H3">
+        <v>660.25</v>
+      </c>
+      <c r="I3">
+        <v>764.95</v>
+      </c>
+      <c r="J3">
+        <v>861.3</v>
+      </c>
+      <c r="K3">
+        <v>952.8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <f>B3-B2</f>
+        <v>-6.1999999999999957</v>
+      </c>
+      <c r="C4">
+        <f t="shared" ref="C4:K4" si="0">C3-C2</f>
+        <v>-21.699999999999989</v>
+      </c>
+      <c r="D4">
+        <f t="shared" si="0"/>
+        <v>-36.800000000000011</v>
+      </c>
+      <c r="E4">
+        <f t="shared" si="0"/>
+        <v>-53.5</v>
+      </c>
+      <c r="F4">
+        <f t="shared" si="0"/>
+        <v>-68.700000000000045</v>
+      </c>
+      <c r="G4">
+        <f t="shared" si="0"/>
+        <v>-85.699999999999932</v>
+      </c>
+      <c r="H4">
+        <f t="shared" si="0"/>
+        <v>-102</v>
+      </c>
+      <c r="I4">
+        <f t="shared" si="0"/>
+        <v>-116.34999999999991</v>
+      </c>
+      <c r="J4">
+        <f t="shared" si="0"/>
+        <v>-134.25</v>
+      </c>
+      <c r="K4">
+        <f t="shared" si="0"/>
+        <v>-152.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5">
+        <f>(ROUND(B4/B2, 2) * 100)</f>
+        <v>-11</v>
+      </c>
+      <c r="C5">
+        <f t="shared" ref="C5:K5" si="1">(ROUND(C4/C2, 2) * 100)</f>
+        <v>-12</v>
+      </c>
+      <c r="D5">
+        <f t="shared" si="1"/>
+        <v>-13</v>
+      </c>
+      <c r="E5">
+        <f t="shared" si="1"/>
+        <v>-13</v>
+      </c>
+      <c r="F5">
+        <f t="shared" si="1"/>
+        <v>-13</v>
+      </c>
+      <c r="G5">
+        <f t="shared" si="1"/>
+        <v>-13</v>
+      </c>
+      <c r="H5">
+        <f t="shared" si="1"/>
+        <v>-13</v>
+      </c>
+      <c r="I5">
+        <f t="shared" si="1"/>
+        <v>-13</v>
+      </c>
+      <c r="J5">
+        <f t="shared" si="1"/>
+        <v>-13</v>
+      </c>
+      <c r="K5">
+        <f t="shared" si="1"/>
+        <v>-14.000000000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>